<commit_message>
Add gitignore and update data
</commit_message>
<xml_diff>
--- a/geosports_history.xlsx
+++ b/geosports_history.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,25 +481,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>86.3</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>93.40000000000001</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>95.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>70.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>258.8</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>896.3</v>
+        <v>945</v>
       </c>
       <c r="J2" t="n">
         <v>945</v>
@@ -511,32 +511,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>johnson5</t>
+          <t>pparril</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>85.8</v>
+        <v>83.5</v>
       </c>
       <c r="E3" t="n">
-        <v>85.8</v>
+        <v>83.5</v>
       </c>
       <c r="F3" t="n">
-        <v>85.8</v>
+        <v>83.5</v>
       </c>
       <c r="G3" t="n">
-        <v>85.8</v>
+        <v>83.5</v>
       </c>
       <c r="H3" t="n">
-        <v>85.8</v>
+        <v>83.5</v>
       </c>
       <c r="I3" t="n">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="J3" t="n">
-        <v>947</v>
+        <v>944</v>
       </c>
     </row>
     <row r="4">
@@ -549,25 +549,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>82.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="E4" t="n">
-        <v>83.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>94.3</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
-        <v>69.5</v>
+        <v>75</v>
       </c>
       <c r="H4" t="n">
-        <v>247.2</v>
+        <v>75</v>
       </c>
       <c r="I4" t="n">
-        <v>891.3</v>
+        <v>926</v>
       </c>
       <c r="J4" t="n">
         <v>926</v>
@@ -579,32 +579,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pparril</t>
+          <t>kadrids</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>64.59999999999999</v>
+        <v>55.5</v>
       </c>
       <c r="E5" t="n">
-        <v>64.59999999999999</v>
+        <v>55.5</v>
       </c>
       <c r="F5" t="n">
-        <v>90.59999999999999</v>
+        <v>55.5</v>
       </c>
       <c r="G5" t="n">
-        <v>38.6</v>
+        <v>55.5</v>
       </c>
       <c r="H5" t="n">
-        <v>129.2</v>
+        <v>55.5</v>
       </c>
       <c r="I5" t="n">
-        <v>825.5</v>
+        <v>894</v>
       </c>
       <c r="J5" t="n">
-        <v>959</v>
+        <v>894</v>
       </c>
     </row>
     <row r="6">
@@ -613,32 +613,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>kadrids</t>
+          <t>JonahL</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>54.4</v>
+        <v>50.8</v>
       </c>
       <c r="E6" t="n">
-        <v>42.3</v>
+        <v>50.8</v>
       </c>
       <c r="F6" t="n">
-        <v>92.7</v>
+        <v>50.8</v>
       </c>
       <c r="G6" t="n">
-        <v>28.1</v>
+        <v>50.8</v>
       </c>
       <c r="H6" t="n">
-        <v>163.1</v>
+        <v>50.8</v>
       </c>
       <c r="I6" t="n">
-        <v>859.7</v>
+        <v>887</v>
       </c>
       <c r="J6" t="n">
-        <v>894</v>
+        <v>887</v>
       </c>
     </row>
     <row r="7">
@@ -647,32 +647,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Spy</t>
+          <t>jbarn11</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>52.2</v>
+        <v>44.2</v>
       </c>
       <c r="E7" t="n">
-        <v>52.2</v>
+        <v>44.2</v>
       </c>
       <c r="F7" t="n">
-        <v>68</v>
+        <v>44.2</v>
       </c>
       <c r="G7" t="n">
-        <v>36.5</v>
+        <v>44.2</v>
       </c>
       <c r="H7" t="n">
-        <v>104.5</v>
+        <v>44.2</v>
       </c>
       <c r="I7" t="n">
-        <v>802.5</v>
+        <v>877</v>
       </c>
       <c r="J7" t="n">
-        <v>917</v>
+        <v>877</v>
       </c>
     </row>
     <row r="8">
@@ -685,28 +685,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>47.6</v>
+        <v>37.7</v>
       </c>
       <c r="E8" t="n">
-        <v>65.09999999999999</v>
+        <v>37.7</v>
       </c>
       <c r="F8" t="n">
-        <v>65.7</v>
+        <v>37.7</v>
       </c>
       <c r="G8" t="n">
-        <v>11.9</v>
+        <v>37.7</v>
       </c>
       <c r="H8" t="n">
-        <v>142.7</v>
+        <v>37.7</v>
       </c>
       <c r="I8" t="n">
-        <v>841</v>
+        <v>867</v>
       </c>
       <c r="J8" t="n">
-        <v>913</v>
+        <v>867</v>
       </c>
     </row>
     <row r="9">
@@ -715,270 +715,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>djeckma</t>
+          <t>johnson7</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>42.3</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>42.3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>42.3</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>42.3</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>42.3</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>699</v>
+        <v>746</v>
       </c>
       <c r="J9" t="n">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Jules</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="F10" t="n">
-        <v>59.7</v>
-      </c>
-      <c r="G10" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="H10" t="n">
-        <v>76.3</v>
-      </c>
-      <c r="I10" t="n">
-        <v>774</v>
-      </c>
-      <c r="J10" t="n">
-        <v>906</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>JonahL</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="E11" t="n">
-        <v>32.7</v>
-      </c>
-      <c r="F11" t="n">
-        <v>69.2</v>
-      </c>
-      <c r="G11" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="H11" t="n">
-        <v>107.5</v>
-      </c>
-      <c r="I11" t="n">
-        <v>817.3</v>
-      </c>
-      <c r="J11" t="n">
-        <v>887</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>cartert</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="E12" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="F12" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="G12" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="H12" t="n">
-        <v>70.59999999999999</v>
-      </c>
-      <c r="I12" t="n">
-        <v>756.5</v>
-      </c>
-      <c r="J12" t="n">
-        <v>912</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>jbarn11</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="E13" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="F13" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="G13" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="H13" t="n">
-        <v>97.59999999999999</v>
-      </c>
-      <c r="I13" t="n">
-        <v>817.3</v>
-      </c>
-      <c r="J13" t="n">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Meghan</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="E14" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="F14" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="G14" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="H14" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="I14" t="n">
-        <v>657</v>
-      </c>
-      <c r="J14" t="n">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>andrewf3</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="E15" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="F15" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="G15" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="H15" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="I15" t="n">
-        <v>621</v>
-      </c>
-      <c r="J15" t="n">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>andrewf2</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="I16" t="n">
-        <v>784</v>
-      </c>
-      <c r="J16" t="n">
-        <v>784</v>
+        <v>746</v>
       </c>
     </row>
   </sheetData>
@@ -992,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1003,16 +765,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>8/31/26</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>9/1/26</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>9/2/26</t>
         </is>
       </c>
@@ -1020,214 +772,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JonahL</t>
+          <t>kunalrs</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>750</v>
-      </c>
-      <c r="C2" t="n">
-        <v>815</v>
-      </c>
-      <c r="D2" t="n">
-        <v>887</v>
+        <v>945</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>pparril</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>642</v>
-      </c>
-      <c r="C3" t="n">
-        <v>906</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>944</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spy</t>
+          <t>Tomh</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>688</v>
-      </c>
-      <c r="C4" t="n">
-        <v>917</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>926</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomh</t>
+          <t>kadrids</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>829</v>
-      </c>
-      <c r="C5" t="n">
-        <v>919</v>
-      </c>
-      <c r="D5" t="n">
-        <v>926</v>
+        <v>894</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ZZ</t>
+          <t>JonahL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>743</v>
-      </c>
-      <c r="C6" t="n">
-        <v>913</v>
-      </c>
-      <c r="D6" t="n">
-        <v>867</v>
+        <v>887</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>andrewf3</t>
+          <t>jbarn11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>621</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+        <v>877</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cartert</t>
+          <t>ZZ</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>601</v>
-      </c>
-      <c r="C8" t="n">
-        <v>912</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>867</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>djeckma</t>
+          <t>johnson7</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>699</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>jbarn11</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>707</v>
-      </c>
-      <c r="C10" t="n">
-        <v>868</v>
-      </c>
-      <c r="D10" t="n">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>kadrids</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>820</v>
-      </c>
-      <c r="C11" t="n">
-        <v>865</v>
-      </c>
-      <c r="D11" t="n">
-        <v>894</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>kunalrs</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>824</v>
-      </c>
-      <c r="C12" t="n">
-        <v>920</v>
-      </c>
-      <c r="D12" t="n">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>pparril</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>692</v>
-      </c>
-      <c r="C13" t="n">
-        <v>959</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Meghan</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>657</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>johnson5</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="n">
-        <v>947</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>andrewf2</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="n">
-        <v>784</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>746</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1240,7 +860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1251,16 +871,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>8/31/26</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>9/1/26</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>9/2/26</t>
         </is>
       </c>
@@ -1268,214 +878,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JonahL</t>
+          <t>kunalrs</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69.2</v>
-      </c>
-      <c r="C2" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.7</v>
+        <v>83.90000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>pparril</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="C3" t="n">
-        <v>59.7</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>83.5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spy</t>
+          <t>Tomh</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="C4" t="n">
-        <v>68</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>75</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomh</t>
+          <t>kadrids</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>94.3</v>
-      </c>
-      <c r="C5" t="n">
-        <v>69.5</v>
-      </c>
-      <c r="D5" t="n">
-        <v>83.40000000000001</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ZZ</t>
+          <t>JonahL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="C6" t="n">
-        <v>65.09999999999999</v>
-      </c>
-      <c r="D6" t="n">
-        <v>11.9</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>andrewf3</t>
+          <t>jbarn11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+        <v>44.2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cartert</t>
+          <t>ZZ</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="C8" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>37.7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>djeckma</t>
+          <t>johnson7</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>jbarn11</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="C10" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="D10" t="n">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>kadrids</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>92.7</v>
-      </c>
-      <c r="C11" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="D11" t="n">
-        <v>42.3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>kunalrs</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>93.40000000000001</v>
-      </c>
-      <c r="C12" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="D12" t="n">
-        <v>95.2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>pparril</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="C13" t="n">
-        <v>90.59999999999999</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Meghan</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>johnson5</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>andrewf2</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1488,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1531,76 +1009,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8/31/26</t>
+          <t>9/2/26</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>713.3</v>
+        <v>885.75</v>
       </c>
       <c r="D2" t="n">
-        <v>73.40000000000001</v>
+        <v>59.74058503228773</v>
       </c>
       <c r="E2" t="n">
-        <v>699</v>
+        <v>890.5</v>
       </c>
       <c r="F2" t="n">
-        <v>829</v>
+        <v>945</v>
       </c>
       <c r="G2" t="n">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>9/1/26</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>12</v>
-      </c>
-      <c r="C3" t="n">
-        <v>893.8</v>
-      </c>
-      <c r="D3" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="E3" t="n">
-        <v>912.5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>959</v>
-      </c>
-      <c r="G3" t="n">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>9/2/26</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" t="n">
-        <v>899.3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>890.5</v>
-      </c>
-      <c r="F4" t="n">
-        <v>945</v>
-      </c>
-      <c r="G4" t="n">
-        <v>867</v>
+        <v>746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>